<commit_message>
Publish Montemor_2021_JWCH, Crestuma_2009_MAR, Poznan_2009_WC
</commit_message>
<xml_diff>
--- a/events/Crestuma_2009_MAR/Crestuma_2009_MAR_Results.xlsx
+++ b/events/Crestuma_2009_MAR/Crestuma_2009_MAR_Results.xlsx
@@ -4284,11 +4284,6 @@
           <t>01:30:31.100</t>
         </is>
       </c>
-      <c r="R63" t="inlineStr">
-        <is>
-          <t>129697</t>
-        </is>
-      </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
@@ -19873,7 +19868,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D132"/>
+  <dimension ref="A1:D131"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -22758,28 +22753,6 @@
         </is>
       </c>
     </row>
-    <row r="132">
-      <c r="A132" t="inlineStr">
-        <is>
-          <t>129697</t>
-        </is>
-      </c>
-      <c r="B132" t="inlineStr">
-        <is>
-          <t>Diogo</t>
-        </is>
-      </c>
-      <c r="C132" t="inlineStr">
-        <is>
-          <t>FERREIRA</t>
-        </is>
-      </c>
-      <c r="D132" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Publish Crestuma_2009_MAR, Halifax_2009_WCH, Moscow_2009_JWCH, Poznan_2009_WC, Racice_2009_WC, Szeged_2009_WC
</commit_message>
<xml_diff>
--- a/events/Crestuma_2009_MAR/Crestuma_2009_MAR_Results.xlsx
+++ b/events/Crestuma_2009_MAR/Crestuma_2009_MAR_Results.xlsx
@@ -4519,6 +4519,11 @@
       <c r="L67" t="n">
         <v>68</v>
       </c>
+      <c r="R67" t="inlineStr">
+        <is>
+          <t>47426</t>
+        </is>
+      </c>
       <c r="X67" t="inlineStr">
         <is>
           <t>DNF</t>
@@ -11882,6 +11887,11 @@
       </c>
       <c r="L189" t="n">
         <v>190</v>
+      </c>
+      <c r="R189" t="inlineStr">
+        <is>
+          <t>47426</t>
+        </is>
       </c>
       <c r="X189" t="inlineStr">
         <is>
@@ -19868,7 +19878,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D131"/>
+  <dimension ref="A1:D132"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -22753,6 +22763,28 @@
         </is>
       </c>
     </row>
+    <row r="132">
+      <c r="A132" t="inlineStr">
+        <is>
+          <t>47426</t>
+        </is>
+      </c>
+      <c r="B132" t="inlineStr">
+        <is>
+          <t>Henrik</t>
+        </is>
+      </c>
+      <c r="C132" t="inlineStr">
+        <is>
+          <t>VASBAYAI</t>
+        </is>
+      </c>
+      <c r="D132" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>